<commit_message>
Update AI insights - דלק
</commit_message>
<xml_diff>
--- a/risks_ai_insights.xlsx
+++ b/risks_ai_insights.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -508,6 +508,41 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>דלק</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>__full_analysis__</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>**דוח סיכונים - פרויקט "דלק"**
+**1. תמונת מצב:**
+פרויקט "דלק" מתמודד עם סיכונים קריטיים הנובעים מתלות במשאב יחיד, בעיות תקשורת ותלות טכנית, העלולים לפגוע באופן משמעותי בהתקדמותו ובהצלחתו.
+**2. 3 סיכונים דחופים:**
+*   **תלות קריטית במפתחת יחידה (הסתברות 5/5, השפעה 5/5):** הסיכון הגבוה ביותר, שכן היעדר גיבוי ידע מהווה נקודת כשל קריטית. כל אירוע המשפיע על זמינותה עלול להשבית את הפרויקט לחלוטין.
+*   **עומס לא צפוי על המפתחת (הסתברות 4/5, השפעה 4/5):** מחייבות פוטנציאליות של המפתחת בפרויקטים אחרים עלולות לגרום לעיכובים קשים בלוחות הזמנים, ולהפחית את יעילות העבודה.
+*   **הזמנות עבודה לא מתחדשות בזמן (הסתברות 4/5, השפעה 4/5):** פערים בהתחדשות הזמנות העבודה עלולים להביא להפסקת כיסוי כספי, פגיעה ישירה בתקציב הפרויקט ובאפשרויות הפעולה שלו.
+**3. דפוסים:**
+*   **"צוואר בקבוק" של משאב יחיד:** תלות קריטית במפתחת יחידה וחשש מעומס עליה מצביעים על ריכוזיות קיצונית של ידע ותפוקה באדם יחיד.
+*   **פערים בתקשורת ותיאום:** קשר חלש מול הלקוח והצורך בתזכורות חוזרות להזמנות עבודה מעידים על חוסר בהירות ובתהליכי עבודה מסודרים אל מול הלקוח.
+*   **חוסר יציבות פנימית ותלות חיצונית:** תלות בממשקי ליבה של הלקוח, יחד עם הסיכון שהם ישתנו, יוצרת פגיעות חיצונית הדורשת גמישות ומוכנות לשינויים, אשר כרגע אינה נתמכת על ידי יציבות פנימית.
+**4. המלצות מיידיות:**
+*   **הכשרת מפתחת גיבוי והעברת ידע:** התחילו באופן מיידי תהליך של העברת ידע ממוקדת והכשרת מפתח נוסף או חליפי, על מנת לפזר את הסיכון של תלות במפתחת יחידה.
+*   **שיפור תהליכי תקשורת ותיאום מול הלקוח:** הגדירו נקודות מפגש קבועות, הפכו את התקשורת לפרואקטיבית, וסדרו תהליך אוטומטי/חצי-אוטומטי לחידוש הזמנות עבודה כדי למנוע הפסקות בכיסוי כספי.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>12/05/2026 18:44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>